<commit_message>
Add 'Bills (Paid & Unpaid)' report support
Introduce a dedicated 'Bills (Paid & Unpaid)' report view and wire it through client and server. UI: update sidebar labels, rename tab label, add Invoice No + Invoice Date nowrap columns and skeleton placeholders in Expense/Bills list pages. Server: add report-scope handling, new BILLS_DETAIL_HEADERS, isBillsReport helper, payment status formatter, adjust monthly report rows/totals and choose headers/totals/title for bills. Excel/PDF generators: include fills, widths and column rules for bill-specific columns. Add test assertions in test-excel-export and update sample xlsx fixture.
</commit_message>
<xml_diff>
--- a/server/tmp/mer-detail-test.xlsx
+++ b/server/tmp/mer-detail-test.xlsx
@@ -8,15 +8,15 @@
     <sheet sheetId="2" name="Summary" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'June'!$1:$9</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Summary'!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'June'!$1:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Summary'!$1:$7</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <r>
       <rPr>
@@ -26,16 +26,6 @@
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">BILLP
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <color rgb="FF000000"/>
-        <sz val="14"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">GST No: 19AALFB4917G1ZB
 </t>
     </r>
     <r>
@@ -55,125 +45,196 @@
         <sz val="14"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t>CIN No: U12345WB2020PTC123456</t>
+      <t xml:space="preserve">CIN No: U12345WB2020PTC123456
+</t>
     </r>
-  </si>
-  <si>
-    <t>Monthly Expense Report | June'2025</t>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>GST No: 19AALFB4917G1ZB</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>BILLP</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> - MONTHLY EXPENSE REPORT COMBINED</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFEF4444"/>
+        <sz val="24"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>JUN'2025</t>
+    </r>
+  </si>
+  <si>
+    <t>S.No</t>
+  </si>
+  <si>
+    <t>Expense No</t>
+  </si>
+  <si>
+    <t>Invoice Date</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Co Name</t>
+  </si>
+  <si>
+    <t>Head of Expense</t>
+  </si>
+  <si>
+    <t>Particulars</t>
+  </si>
+  <si>
+    <t>Expense Type</t>
+  </si>
+  <si>
+    <t>Net Amount</t>
+  </si>
+  <si>
+    <t>Total GST</t>
+  </si>
+  <si>
+    <t>TDS</t>
+  </si>
+  <si>
+    <t>Gross Amount</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
+  </si>
+  <si>
+    <t>Approval Status</t>
+  </si>
+  <si>
+    <t>EXP/BSIBPL/26-27/Jun/001</t>
+  </si>
+  <si>
+    <t>15-06-2025</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>Baid Inbest Llp</t>
+  </si>
+  <si>
+    <t>Test Co</t>
+  </si>
+  <si>
+    <t>Office Supplies</t>
+  </si>
+  <si>
+    <t>Printer paper and toner cartridges</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Bank</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>EXP/BSIBPL/26-27/Jun/002</t>
+  </si>
+  <si>
+    <t>20-06-2025</t>
+  </si>
+  <si>
+    <t>Test Co 2</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Cab fare</t>
+  </si>
+  <si>
+    <t>UPI</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>2 entries</t>
+  </si>
+  <si>
+    <t>TOTAL AMOUNT</t>
+  </si>
+  <si>
+    <t>Amount (in words): Rupees One Crore Fifteen Lakh Thirty Five Thousand Seven Hundred Sixty Four Only</t>
   </si>
   <si>
     <t>MER/BILLP/HQ/25-26/Jun</t>
   </si>
   <si>
-    <t>S.No</t>
-  </si>
-  <si>
-    <t>Expense No</t>
-  </si>
-  <si>
-    <t>Invoice Date</t>
-  </si>
-  <si>
-    <t>Month</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Co Name</t>
-  </si>
-  <si>
-    <t>Head of Expense</t>
-  </si>
-  <si>
-    <t>Particulars</t>
-  </si>
-  <si>
-    <t>Expense Type</t>
-  </si>
-  <si>
-    <t>Net Amount</t>
-  </si>
-  <si>
-    <t>Total GST</t>
-  </si>
-  <si>
-    <t>TDS</t>
-  </si>
-  <si>
-    <t>Gross Amount</t>
-  </si>
-  <si>
-    <t>Payment Method</t>
-  </si>
-  <si>
-    <t>Approval Status</t>
-  </si>
-  <si>
-    <t>EXP/BSIBPL/26-27/Jun/001</t>
-  </si>
-  <si>
-    <t>15-06-2025</t>
-  </si>
-  <si>
-    <t>June</t>
-  </si>
-  <si>
-    <t>Baid Inbest Llp</t>
-  </si>
-  <si>
-    <t>Test Co</t>
-  </si>
-  <si>
-    <t>Office Supplies</t>
-  </si>
-  <si>
-    <t>Printer paper and toner cartridges</t>
-  </si>
-  <si>
-    <t>Revenue</t>
-  </si>
-  <si>
-    <t>Bank</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>EXP/BSIBPL/26-27/Jun/002</t>
-  </si>
-  <si>
-    <t>20-06-2025</t>
-  </si>
-  <si>
-    <t>Test Co 2</t>
-  </si>
-  <si>
-    <t>Travel</t>
-  </si>
-  <si>
-    <t>Cab fare</t>
-  </si>
-  <si>
-    <t>UPI</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Totals</t>
-  </si>
-  <si>
-    <t>2 entries</t>
-  </si>
-  <si>
-    <t>TOTAL AMOUNT</t>
-  </si>
-  <si>
-    <t>Amount (in words): Rupees One Crore Fifteen Lakh Thirty Five Thousand Seven Hundred Sixty Four Only</t>
-  </si>
-  <si>
-    <t>6th Floor, Suite No 608 And 609, Ashoka House, 3a, Hare St, B.b.d. Bagh, Kolkata, West Bengal, 700001, India</t>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Internal Documents</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FF000000"/>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color rgb="FFEF4444"/>
+        <sz val="12"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Accounts Department</t>
+    </r>
   </si>
   <si>
     <t>MER Summary Report</t>
@@ -198,22 +259,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot; #,##0"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -228,36 +279,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF047857"/>
-      <sz val="12"/>
+      <sz val="13"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFB91C1C"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF1F2937"/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF166534"/>
-      <sz val="14"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF7F1D1D"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
       <name val="Calibri"/>
     </font>
@@ -275,12 +302,17 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -294,27 +326,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEFF3FA"/>
+        <fgColor rgb="FFC5DCE8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEE2E2"/>
+        <fgColor rgb="FF86B8CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF13AFCD"/>
       </patternFill>
     </fill>
   </fills>
@@ -345,7 +367,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -353,66 +375,57 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -922,15 +935,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:V20"/>
+  <dimension ref="B1:V18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="10" width="36" customWidth="1"/>
@@ -1064,7 +1076,7 @@
       <c r="V5" s="2"/>
     </row>
     <row r="6" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="7" ht="32" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
@@ -1089,319 +1101,296 @@
       <c r="U7" s="3"/>
       <c r="V7" s="3"/>
     </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="8" ht="36" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="4"/>
-      <c r="V8" s="4"/>
-    </row>
-    <row r="11" ht="36" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="H8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="I8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="J8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="K8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="L8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="M8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="N8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="O8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="P8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B9" s="6">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B12" s="7">
-        <v>1</v>
-      </c>
-      <c r="C12" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="E9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="F9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="H9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="I9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="J9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="K9" s="9">
+        <v>9876543</v>
+      </c>
+      <c r="L9" s="9">
+        <v>1777777</v>
+      </c>
+      <c r="M9" s="10">
+        <v>123456</v>
+      </c>
+      <c r="N9" s="9">
+        <v>11530864</v>
+      </c>
+      <c r="O9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="K12" s="10">
-        <v>9876543</v>
-      </c>
-      <c r="L12" s="11">
+      <c r="P9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B10" s="6">
+        <v>2</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="9">
+        <v>5000</v>
+      </c>
+      <c r="L10" s="9">
+        <v>0</v>
+      </c>
+      <c r="M10" s="10">
+        <v>100</v>
+      </c>
+      <c r="N10" s="9">
+        <v>4900</v>
+      </c>
+      <c r="O10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="K11" s="14">
+        <v>9881543</v>
+      </c>
+      <c r="L11" s="14">
         <v>1777777</v>
       </c>
-      <c r="M12" s="12">
-        <v>123456</v>
-      </c>
-      <c r="N12" s="13">
-        <v>11530864</v>
-      </c>
-      <c r="O12" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="P12" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="7">
-        <v>2</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I13" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="K13" s="10">
-        <v>5000</v>
-      </c>
-      <c r="L13" s="11">
-        <v>0</v>
-      </c>
-      <c r="M13" s="12">
-        <v>100</v>
-      </c>
-      <c r="N13" s="13">
-        <v>4900</v>
-      </c>
-      <c r="O13" s="7" t="s">
+      <c r="M11" s="14">
+        <v>123556</v>
+      </c>
+      <c r="N11" s="14">
+        <v>11535764</v>
+      </c>
+      <c r="O11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="P13" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-    </row>
-    <row r="14" ht="28" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="I14" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="J14" s="14" t="s">
+      <c r="P11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="5"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B12" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="K14" s="17">
-        <v>9881543</v>
-      </c>
-      <c r="L14" s="18">
-        <v>1777777</v>
-      </c>
-      <c r="M14" s="19">
-        <v>123556</v>
-      </c>
-      <c r="N14" s="17">
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="16">
         <v>11535764</v>
       </c>
-      <c r="O14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="P14" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="6"/>
-    </row>
-    <row r="15" ht="26" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B15" s="20" t="s">
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B14" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
-      <c r="O15" s="20"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20"/>
-      <c r="T15" s="20"/>
-      <c r="U15" s="20"/>
-      <c r="V15" s="21">
-        <v>11535764</v>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B17" s="22" t="s">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="17"/>
+      <c r="V14" s="17"/>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B18" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="22"/>
-      <c r="R17" s="22"/>
-      <c r="S17" s="22"/>
-      <c r="T17" s="22"/>
-      <c r="U17" s="22"/>
-      <c r="V17" s="22"/>
-    </row>
-    <row r="20" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B20" s="23" t="s">
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="23"/>
-      <c r="N20" s="23"/>
-      <c r="O20" s="23"/>
-      <c r="P20" s="23"/>
-      <c r="Q20" s="23"/>
-      <c r="R20" s="23"/>
-      <c r="S20" s="23"/>
-      <c r="T20" s="23"/>
-      <c r="U20" s="23"/>
-      <c r="V20" s="23"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="19"/>
+      <c r="Q18" s="19"/>
+      <c r="R18" s="19"/>
+      <c r="S18" s="19"/>
+      <c r="T18" s="19"/>
+      <c r="U18" s="19"/>
+      <c r="V18" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1409,10 +1398,10 @@
     <mergeCell ref="I1:O5"/>
     <mergeCell ref="P1:V5"/>
     <mergeCell ref="B7:V7"/>
-    <mergeCell ref="B8:V8"/>
-    <mergeCell ref="B15:U15"/>
-    <mergeCell ref="B17:V17"/>
-    <mergeCell ref="B20:V20"/>
+    <mergeCell ref="B12:U12"/>
+    <mergeCell ref="B14:V14"/>
+    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="M18:V18"/>
   </mergeCells>
   <pageMargins left="0.21" right="0.21" top="0.21" bottom="0.21" header="0.21" footer="0.21"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
@@ -1425,14 +1414,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:V19"/>
+  <dimension ref="B1:V14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="4" width="10" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
     <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="6" max="6" width="8" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
@@ -1568,225 +1556,199 @@
       <c r="V5" s="2"/>
     </row>
     <row r="6" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+    <row r="7" ht="32" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B7" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
-    </row>
-    <row r="10" ht="36" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="20"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="20"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="20"/>
+      <c r="N7" s="20"/>
+      <c r="O7" s="20"/>
+      <c r="P7" s="20"/>
+      <c r="Q7" s="20"/>
+      <c r="R7" s="20"/>
+      <c r="S7" s="20"/>
+      <c r="T7" s="20"/>
+      <c r="U7" s="20"/>
+      <c r="V7" s="20"/>
+    </row>
+    <row r="8" ht="36" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="6"/>
-      <c r="V10" s="6"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+    </row>
+    <row r="9" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="6">
+        <v>9881543</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+    </row>
+    <row r="10" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="6">
+        <v>11535764</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
     </row>
     <row r="11" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="7">
-        <v>9881543</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-      <c r="U11" s="6"/>
-      <c r="V11" s="6"/>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B12" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="7">
+      <c r="B11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="5"/>
+      <c r="V11" s="5"/>
+    </row>
+    <row r="12" ht="26" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B12" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="16">
         <v>11535764</v>
       </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
-      <c r="V12" s="6"/>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" s="7">
-        <v>2</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
-      <c r="V13" s="6"/>
-    </row>
-    <row r="14" ht="26" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B14" s="20" t="s">
+    </row>
+    <row r="14" ht="24" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B14" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="20"/>
-      <c r="N14" s="20"/>
-      <c r="O14" s="20"/>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="20"/>
-      <c r="S14" s="20"/>
-      <c r="T14" s="20"/>
-      <c r="U14" s="20"/>
-      <c r="V14" s="21">
-        <v>11535764</v>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B16" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
-      <c r="R16" s="22"/>
-      <c r="S16" s="22"/>
-      <c r="T16" s="22"/>
-      <c r="U16" s="22"/>
-      <c r="V16" s="22"/>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B19" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="23"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="23"/>
-      <c r="T19" s="23"/>
-      <c r="U19" s="23"/>
-      <c r="V19" s="23"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="17"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
+      <c r="U14" s="17"/>
+      <c r="V14" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="B1:H5"/>
     <mergeCell ref="I1:O5"/>
     <mergeCell ref="P1:V5"/>
     <mergeCell ref="B7:V7"/>
-    <mergeCell ref="B14:U14"/>
-    <mergeCell ref="B16:V16"/>
-    <mergeCell ref="B19:V19"/>
+    <mergeCell ref="B12:U12"/>
+    <mergeCell ref="B14:V14"/>
   </mergeCells>
   <pageMargins left="0.21" right="0.21" top="0.21" bottom="0.21" header="0.21" footer="0.21"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>

</xml_diff>